<commit_message>
PDF de entrega del 30/10 completo: sorteo oficial, plan de línea base, 3 preguntas, anexos con enlaces; guía de medición
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05 - Ciclos y bitacora/29102026_01_Bitacora_v2.xlsx
+++ b/05 - Ciclos y bitacora/29102026_01_Bitacora_v2.xlsx
@@ -787,14 +787,28 @@
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr"/>
-      <c r="C2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
       <c r="D2" s="7" t="inlineStr"/>
       <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Ana Sofía Arango Yanza y Juan José Arias Chacua</t>
+        </is>
+      </c>
       <c r="G2" s="6" t="inlineStr"/>
       <c r="H2" s="6" t="inlineStr"/>
-      <c r="I2" s="6" t="inlineStr"/>
-      <c r="J2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>ninguna</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>30102026</v>
+      </c>
       <c r="K2" s="6" t="inlineStr"/>
       <c r="L2" s="6" t="inlineStr"/>
       <c r="M2" s="6" t="inlineStr"/>
@@ -807,14 +821,28 @@
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr"/>
-      <c r="C3" s="8" t="inlineStr"/>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
       <c r="D3" s="9" t="inlineStr"/>
       <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="8" t="inlineStr"/>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Ana Sofía Arango Yanza y Juan José Arias Chacua</t>
+        </is>
+      </c>
       <c r="G3" s="8" t="inlineStr"/>
       <c r="H3" s="8" t="inlineStr"/>
-      <c r="I3" s="8" t="inlineStr"/>
-      <c r="J3" s="8" t="inlineStr"/>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>ninguna</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>30102026</v>
+      </c>
       <c r="K3" s="8" t="inlineStr"/>
       <c r="L3" s="8" t="inlineStr"/>
       <c r="M3" s="8" t="inlineStr"/>
@@ -827,14 +855,28 @@
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="inlineStr"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
       <c r="D4" s="7" t="inlineStr"/>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Ana Sofía Arango Yanza y Juan José Arias Chacua</t>
+        </is>
+      </c>
       <c r="G4" s="6" t="inlineStr"/>
       <c r="H4" s="6" t="inlineStr"/>
-      <c r="I4" s="6" t="inlineStr"/>
-      <c r="J4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>ninguna</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>30102026</v>
+      </c>
       <c r="K4" s="6" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr"/>
       <c r="M4" s="6" t="inlineStr"/>
@@ -1129,8 +1171,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr"/>
-      <c r="F2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G2" s="6" t="inlineStr"/>
       <c r="H2" s="6" t="inlineStr"/>
       <c r="I2" s="7" t="n"/>
@@ -1182,8 +1232,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr"/>
-      <c r="F3" s="8" t="inlineStr"/>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G3" s="8" t="inlineStr"/>
       <c r="H3" s="8" t="inlineStr"/>
       <c r="I3" s="9" t="n"/>
@@ -1235,8 +1293,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 1</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Ana Sofía</t>
+        </is>
+      </c>
       <c r="G4" s="6" t="inlineStr"/>
       <c r="H4" s="6" t="inlineStr"/>
       <c r="I4" s="7" t="n"/>
@@ -1288,8 +1354,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr"/>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Repuesto</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G5" s="8" t="inlineStr"/>
       <c r="H5" s="8" t="inlineStr"/>
       <c r="I5" s="9" t="n"/>
@@ -1341,8 +1415,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="7" t="n"/>
@@ -1394,8 +1476,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Repuesto</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G7" s="8" t="inlineStr"/>
       <c r="H7" s="8" t="inlineStr"/>
       <c r="I7" s="9" t="n"/>
@@ -1447,8 +1537,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 1</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Ana Sofía</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="7" t="n"/>
@@ -1500,8 +1598,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G9" s="8" t="inlineStr"/>
       <c r="H9" s="8" t="inlineStr"/>
       <c r="I9" s="9" t="n"/>
@@ -1553,8 +1659,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="7" t="n"/>
@@ -1606,8 +1720,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Ciclo 2</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Ana Sofía</t>
+        </is>
+      </c>
       <c r="G11" s="8" t="inlineStr"/>
       <c r="H11" s="8" t="inlineStr"/>
       <c r="I11" s="9" t="n"/>
@@ -1659,8 +1781,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 2</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Ana Sofía</t>
+        </is>
+      </c>
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="7" t="n"/>
@@ -1712,8 +1842,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Ciclo 1</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Ana Sofía</t>
+        </is>
+      </c>
       <c r="G13" s="8" t="inlineStr"/>
       <c r="H13" s="8" t="inlineStr"/>
       <c r="I13" s="9" t="n"/>
@@ -1765,8 +1903,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 2</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Juan José</t>
+        </is>
+      </c>
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="7" t="n"/>
@@ -1818,8 +1964,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Ciclo 1</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Juan José</t>
+        </is>
+      </c>
       <c r="G15" s="8" t="inlineStr"/>
       <c r="H15" s="8" t="inlineStr"/>
       <c r="I15" s="9" t="n"/>
@@ -1871,8 +2025,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 1</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Juan José</t>
+        </is>
+      </c>
       <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="7" t="n"/>
@@ -1924,8 +2086,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G17" s="8" t="inlineStr"/>
       <c r="H17" s="8" t="inlineStr"/>
       <c r="I17" s="9" t="n"/>
@@ -1977,8 +2147,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="6" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 2</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Juan José</t>
+        </is>
+      </c>
       <c r="G18" s="6" t="inlineStr"/>
       <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="7" t="n"/>
@@ -2030,8 +2208,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G19" s="8" t="inlineStr"/>
       <c r="H19" s="8" t="inlineStr"/>
       <c r="I19" s="9" t="n"/>
@@ -2083,8 +2269,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 1</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Juan José</t>
+        </is>
+      </c>
       <c r="G20" s="6" t="inlineStr"/>
       <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="7" t="n"/>
@@ -2136,8 +2330,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr"/>
-      <c r="F21" s="8" t="inlineStr"/>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G21" s="8" t="inlineStr"/>
       <c r="H21" s="8" t="inlineStr"/>
       <c r="I21" s="9" t="n"/>
@@ -2189,8 +2391,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G22" s="6" t="inlineStr"/>
       <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="7" t="n"/>
@@ -2242,8 +2452,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Línea base</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Pareja (A y J)</t>
+        </is>
+      </c>
       <c r="G23" s="8" t="inlineStr"/>
       <c r="H23" s="8" t="inlineStr"/>
       <c r="I23" s="9" t="n"/>
@@ -2295,8 +2513,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Ciclo 2</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Ana Sofía</t>
+        </is>
+      </c>
       <c r="G24" s="6" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="7" t="n"/>
@@ -2348,8 +2574,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr"/>
-      <c r="F25" s="8" t="inlineStr"/>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Ciclo 2</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Juan José</t>
+        </is>
+      </c>
       <c r="G25" s="8" t="inlineStr"/>
       <c r="H25" s="8" t="inlineStr"/>
       <c r="I25" s="9" t="n"/>

</xml_diff>